<commit_message>
Update clean names and build portal
</commit_message>
<xml_diff>
--- a/leads_advocacia_campinas.xlsx
+++ b/leads_advocacia_campinas.xlsx
@@ -491,7 +491,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MAP Advocacia</t>
+          <t>Map Advocacia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -529,10 +529,8 @@
           <t>(19) 3342-9460</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>551933429460</t>
-        </is>
+      <c r="I2" t="n">
+        <v>551933429460</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -569,7 +567,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10 MELHORES Escritrios de Advocacia em Campin</t>
+          <t>10 Melhores Escritrios de Advocacia em C</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,7 +641,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Advocacia em Campinas SP (2026)</t>
+          <t>Advocacia em Campinas Sp (2026)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -717,7 +715,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Os Melhores Advogados de Campinas</t>
+          <t>Os Melhores Advogados de</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -791,7 +789,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Escritrio de Advocacia Direito Previdencirio</t>
+          <t>Escritrio de Advocacia Direito Previdenc</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -865,7 +863,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Advocacia Campinas</t>
+          <t>Advocacia</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -903,10 +901,8 @@
           <t>(19) 3212-1674</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>551932121674</t>
-        </is>
+      <c r="I7" t="n">
+        <v>551932121674</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -943,7 +939,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Leads de Assistncias tcnicas em Campinas</t>
+          <t>Leads de Assistncias Tcnicas</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1017,7 +1013,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Consani Advocacia Campinas</t>
+          <t>Consani Advocacia</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1055,10 +1051,8 @@
           <t>(19) 99294-6366</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>5519992946366</t>
-        </is>
+      <c r="I9" t="n">
+        <v>5519992946366</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1095,7 +1089,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kontato para Advocacia em Campinas SP</t>
+          <t>Kontato para Advocacia</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1133,10 +1127,8 @@
           <t>(19) 3256-2415</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>551932562415</t>
-        </is>
+      <c r="I10" t="n">
+        <v>551932562415</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1173,7 +1165,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mem de S Advogado em Campinas</t>
+          <t>Mem de S Advogado</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1247,7 +1239,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GFJr. Advocacia &amp; consultoria</t>
+          <t>Gfjr. Advocacia &amp; Consultoria</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1285,10 +1277,8 @@
           <t>(19) 3294-9147</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>551932949147</t>
-        </is>
+      <c r="I12" t="n">
+        <v>551932949147</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -1325,7 +1315,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Advogado Trabalhista em Campinas</t>
+          <t>Advogado Trabalhista</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1363,10 +1353,8 @@
           <t>(19) 3433-7202</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>551934337202</t>
-        </is>
+      <c r="I13" t="n">
+        <v>551934337202</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1403,7 +1391,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10 melhores advogados em direito imobilirio p</t>
+          <t>10 Melhores Advogados em Direito Imobili</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1477,7 +1465,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Compare advogados em Campinas</t>
+          <t>Compare Advogados</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1625,7 +1613,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Advogado Campinas</t>
+          <t>Advogado</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1663,10 +1651,8 @@
           <t>(19) 4062-9893</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>551940629893</t>
-        </is>
+      <c r="I17" t="n">
+        <v>551940629893</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1741,10 +1727,8 @@
           <t>(19) 97155-5272</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>5519971555272</t>
-        </is>
+      <c r="I18" t="n">
+        <v>5519971555272</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1819,10 +1803,8 @@
           <t>(19) 3734-1222</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>551937341222</t>
-        </is>
+      <c r="I19" t="n">
+        <v>551937341222</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1933,7 +1915,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CAASP de Campinas,</t>
+          <t>Caasp de</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2007,7 +1989,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dr. Rafael Nascimento advocacia, Campinas</t>
+          <t>Dr. Rafael Nascimento Advocacia</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2045,10 +2027,8 @@
           <t>(19) 98227-9369</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>5519982279369</t>
-        </is>
+      <c r="I22" t="n">
+        <v>5519982279369</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -2123,10 +2103,8 @@
           <t>(18) 9813-8764</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>551898138764</t>
-        </is>
+      <c r="I23" t="n">
+        <v>551898138764</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -2163,7 +2141,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Karabalis e Martendal Advocacia Campinas So J</t>
+          <t>Karabalis e Martendal Advocacia</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2201,10 +2179,8 @@
           <t>(48) 3375-8470</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>554833758470</t>
-        </is>
+      <c r="I24" t="n">
+        <v>554833758470</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -2241,7 +2217,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Advogados e Escritrios de Advocacia em Campin</t>
+          <t>Advogados e Escritrios de Advocacia em C</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2315,7 +2291,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Advocacia Campinas Sylvia Barbosa em Campinas</t>
+          <t>Advocacia Campinas Sylvia Barbosa</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2353,10 +2329,8 @@
           <t>(19) 99704-4630</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>5519997044630</t>
-        </is>
+      <c r="I26" t="n">
+        <v>5519997044630</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -2505,10 +2479,8 @@
           <t>(11) 3262-0706</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>551132620706</t>
-        </is>
+      <c r="I28" t="n">
+        <v>551132620706</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2583,10 +2555,8 @@
           <t>(19) 9843-0757</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>551998430757</t>
-        </is>
+      <c r="I29" t="n">
+        <v>551998430757</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2735,10 +2705,8 @@
           <t>(19) 3233-6880</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>551932336880</t>
-        </is>
+      <c r="I31" t="n">
+        <v>551932336880</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2923,7 +2891,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Advogados em Campinas</t>
+          <t>Advogados</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2961,10 +2929,8 @@
           <t>(19) 98199-0236</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>5519981990236</t>
-        </is>
+      <c r="I34" t="n">
+        <v>5519981990236</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -3149,7 +3115,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DM Advocacia</t>
+          <t>Dm Advocacia</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3187,10 +3153,8 @@
           <t>(19) 97110-3795</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>5519971103795</t>
-        </is>
+      <c r="I37" t="n">
+        <v>5519971103795</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -3227,7 +3191,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>reas de Atuao</t>
+          <t>Reas de Atuao</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3339,10 +3303,8 @@
           <t>(19) 98812-8079</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>5519988128079</t>
-        </is>
+      <c r="I39" t="n">
+        <v>5519988128079</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -3417,10 +3379,8 @@
           <t>(19) 3307-7147</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>551933077147</t>
-        </is>
+      <c r="I40" t="n">
+        <v>551933077147</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -3457,7 +3417,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>10 Melhores Barbearias em Campinas</t>
+          <t>10 Melhores Barbearias</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3495,10 +3455,8 @@
           <t>(19) 3294-1717</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>551932941717</t>
-        </is>
+      <c r="I41" t="n">
+        <v>551932941717</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -3573,10 +3531,8 @@
           <t>(19) 98604-9825</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>5519986049825</t>
-        </is>
+      <c r="I42" t="n">
+        <v>5519986049825</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -3613,7 +3569,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Barbearia em Campinas</t>
+          <t>Barbearia</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3651,10 +3607,8 @@
           <t>(19) 3238-6122</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>551932386122</t>
-        </is>
+      <c r="I43" t="n">
+        <v>551932386122</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
@@ -3691,7 +3645,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Estao Campinas</t>
+          <t>Estao</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3765,7 +3719,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Barbearia Campinas</t>
+          <t>Barbearia</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">

</xml_diff>